<commit_message>
Added new files and code change
</commit_message>
<xml_diff>
--- a/12601472.xlsx
+++ b/12601472.xlsx
@@ -8,9 +8,9 @@
       <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="C:\Users\SAM\Projects-Code\University-Codes\PYTHON\CA_MINI_PROJECT_1\"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{91938258-1E11-4721-8C04-10A373E4EEEA}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
+  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{BDAD3C86-6812-4DA1-AF5E-D797CD472F3B}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
   <bookViews>
-    <workbookView xWindow="28680" yWindow="-120" windowWidth="20730" windowHeight="11040" tabRatio="500" activeTab="1" xr2:uid="{00000000-000D-0000-FFFF-FFFF00000000}"/>
+    <workbookView xWindow="-110" yWindow="-110" windowWidth="19420" windowHeight="10300" tabRatio="500" activeTab="1" xr2:uid="{00000000-000D-0000-FFFF-FFFF00000000}"/>
   </bookViews>
   <sheets>
     <sheet name="Instructions" sheetId="1" r:id="rId1"/>
@@ -21,7 +21,7 @@
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="214" uniqueCount="105">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="218" uniqueCount="106">
   <si>
     <t>My Data, My Code</t>
   </si>
@@ -336,6 +336,9 @@
   </si>
   <si>
     <t xml:space="preserve">Day went as usual, little bit borring </t>
+  </si>
+  <si>
+    <t>Boring day</t>
   </si>
 </sst>
 </file>
@@ -2972,15 +2975,15 @@
         <v>8</v>
       </c>
       <c r="H40" s="9">
-        <v>119</v>
+        <v>120</v>
       </c>
       <c r="I40" s="10">
         <f t="shared" si="0"/>
-        <v>1034</v>
+        <v>1035</v>
       </c>
       <c r="J40" s="10">
         <f t="shared" si="1"/>
-        <v>406</v>
+        <v>405</v>
       </c>
       <c r="K40" s="11" t="s">
         <v>82</v>
@@ -3018,15 +3021,15 @@
         <v>3</v>
       </c>
       <c r="H41" s="9">
-        <v>119</v>
+        <v>120</v>
       </c>
       <c r="I41" s="10">
         <f t="shared" si="0"/>
-        <v>1137</v>
+        <v>1138</v>
       </c>
       <c r="J41" s="10">
         <f t="shared" si="1"/>
-        <v>303</v>
+        <v>302</v>
       </c>
       <c r="K41" s="11" t="s">
         <v>51</v>
@@ -3064,15 +3067,15 @@
         <v>3</v>
       </c>
       <c r="H42" s="9">
-        <v>119</v>
+        <v>120</v>
       </c>
       <c r="I42" s="10">
         <f t="shared" si="0"/>
-        <v>1094</v>
+        <v>1095</v>
       </c>
       <c r="J42" s="10">
         <f t="shared" si="1"/>
-        <v>346</v>
+        <v>345</v>
       </c>
       <c r="K42" s="11" t="s">
         <v>54</v>
@@ -3110,15 +3113,15 @@
         <v>2</v>
       </c>
       <c r="H43" s="9">
-        <v>119</v>
+        <v>60</v>
       </c>
       <c r="I43" s="10">
         <f t="shared" si="0"/>
-        <v>981</v>
+        <v>922</v>
       </c>
       <c r="J43" s="10">
         <f t="shared" si="1"/>
-        <v>459</v>
+        <v>518</v>
       </c>
       <c r="K43" s="11" t="s">
         <v>54</v>
@@ -3180,26 +3183,50 @@
       </c>
     </row>
     <row r="45" spans="1:14" ht="14.5" customHeight="1" x14ac:dyDescent="0.35">
-      <c r="A45" s="8"/>
-      <c r="B45" s="9"/>
-      <c r="C45" s="9"/>
-      <c r="D45" s="9"/>
-      <c r="E45" s="9"/>
-      <c r="F45" s="9"/>
-      <c r="G45" s="9"/>
-      <c r="H45" s="9"/>
-      <c r="I45" s="10" t="str">
+      <c r="A45" s="8">
+        <v>46286</v>
+      </c>
+      <c r="B45" s="9">
+        <v>420</v>
+      </c>
+      <c r="C45" s="9">
+        <v>30</v>
+      </c>
+      <c r="D45" s="9">
+        <v>60</v>
+      </c>
+      <c r="E45" s="9">
+        <v>120</v>
+      </c>
+      <c r="F45" s="9">
+        <v>300</v>
+      </c>
+      <c r="G45" s="9">
+        <v>6</v>
+      </c>
+      <c r="H45" s="9">
+        <v>90</v>
+      </c>
+      <c r="I45" s="10">
         <f t="shared" si="0"/>
-        <v/>
-      </c>
-      <c r="J45" s="10" t="str">
+        <v>1020</v>
+      </c>
+      <c r="J45" s="10">
         <f t="shared" si="1"/>
-        <v/>
-      </c>
-      <c r="K45" s="11"/>
-      <c r="L45" s="11"/>
-      <c r="M45" s="11"/>
-      <c r="N45" s="12"/>
+        <v>420</v>
+      </c>
+      <c r="K45" s="11" t="s">
+        <v>51</v>
+      </c>
+      <c r="L45" s="11" t="s">
+        <v>59</v>
+      </c>
+      <c r="M45" s="11" t="s">
+        <v>52</v>
+      </c>
+      <c r="N45" s="12" t="s">
+        <v>105</v>
+      </c>
     </row>
     <row r="46" spans="1:14" ht="14.5" customHeight="1" x14ac:dyDescent="0.35">
       <c r="A46" s="8"/>

</xml_diff>